<commit_message>
Update blog database with current Squarespace blog posts
Replace the new-site-only list with a full migration database: 22 posts from
the current www.californiafastener.com Squarespace blog (compiled via search;
the site blocks crawling) on sheet 1, the 2 rebuilt posts on sheet 2, plus a
redirect-mapping column and notes on verifying completeness via the
Squarespace JSON feed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L7SQm2b6jQV6c4Prz3vF39
</commit_message>
<xml_diff>
--- a/California-Fastener-Blog-Database.xlsx
+++ b/California-Fastener-Blog-Database.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Blog Posts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Current site blog (Squarespace)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="New site blog (live)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +34,11 @@
     </font>
     <font>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
@@ -84,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -97,6 +103,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,19 +469,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -490,42 +493,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Current URL (www.californiafastener.com)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>Slug</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>On new site?</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>New live URL (redirect target)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Slug</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Excerpt</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Author</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>OLD site URL (fill in → redirect from)</t>
+          <t>Redirect → new URL (301)</t>
         </is>
       </c>
     </row>
@@ -535,45 +518,21 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Understanding ASTM A193 B7 vs. A193 B16: A Comprehensive Guide</t>
+          <t>Precision Matters: How Custom CNC Fasteners Are Revolutionizing Industrial Manufacturing</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Materials &amp; Grades</t>
+          <t>https://www.californiafastener.com/blog/custom-cnc-fasteners-industrial-manufacturing</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2 min</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>https://californiafastener.com/blog/astm-a193-b7-vs-a193-b16</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>astm-a193-b7-vs-a193-b16</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Dive into the details of ASTM A193 B7 and A193 B16 to understand their differences, applications, and how to make the right choice for your project needs.</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>California Fastener</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr"/>
+          <t>custom-cnc-fasteners-industrial-manufacturing</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -581,45 +540,469 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>How Custom CNC Fasteners Help Engineers Break Design Barriers</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/how-custom-cnc-fasteners-help-engineers-break-design-barriers</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>how-custom-cnc-fasteners-help-engineers-break-design-barriers</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Fast Turnarounds, Tight Tolerances: CNC Capabilities at California Fastener</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/cnc-capabilities-at-california-fastener</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>cnc-capabilities-at-california-fastener</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Low-Volume, High-Precision: When CNC Machining Outperforms Traditional Fastener Manufacturing</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/tlmdtgthiz6l7p30otc7s5dm02khh9</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>tlmdtgthiz6l7p30otc7s5dm02khh9</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>The Ultimate Guide to Stainless Steel Fasteners</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/the-ultimate-guide-to-stainless-steel-fasteners</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>the-ultimate-guide-to-stainless-steel-fasteners</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
           <t>The Ultimate Guide to ASTM F593 Stainless Steel Fasteners</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Materials &amp; Grades</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>3 min</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/the-ultimate-guide-to-astm-f593-stainless-steel-fasteners</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>the-ultimate-guide-to-astm-f593-stainless-steel-fasteners</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>https://californiafastener.com/blog/guide-to-astm-f593-stainless-steel-fasteners</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>guide-to-astm-f593-stainless-steel-fasteners</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>ASTM F593 is a specification that covers the chemical and mechanical requirements for stainless steel bolts, hex cap screws, and studs in diameters ranging from 1/4 inch to 1-1/2 inches inclusive.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>California Fastener</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>The Ultimate Guide to Industrial Anchor Bolts</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/the-ultimate-guide-to-industrial-anchor-bolts</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>the-ultimate-guide-to-industrial-anchor-bolts</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>A Comprehensive Guide to Industrial Fasteners: Types, Materials, and Applications</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/a-comprehensive-guide-to-industrial-fasteners</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>a-comprehensive-guide-to-industrial-fasteners</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>The Comprehensive Guide to ASTM A193 Fasteners</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/guide-to-astm-a193-fasteners</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>guide-to-astm-a193-fasteners</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>The Comprehensive Guide to ASTM A193: Understanding Each Grade</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/the-comprehensive-guide-to-astm-a193-understanding-each-grade</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>the-comprehensive-guide-to-astm-a193-understanding-each-grade</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Ultimate Guide to ASTM A490 Heavy-Hex Bolts — Specs &amp; Uses</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/astm-a490-heavy-hex-bolts-specs-uses</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>astm-a490-heavy-hex-bolts-specs-uses</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>High-Strength Connections: A Guide to ASTM A490 Bolts</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/high-strength-connections-a-guide-to-astm-a490-bolts</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>high-strength-connections-a-guide-to-astm-a490-bolts</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>ASTM A449 Bolts: Versatile Fasteners for General Engineering</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/astm-a449-bolts-versatile-fasteners-for-general-engineering</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>astm-a449-bolts-versatile-fasteners-for-general-engineering</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Exploring ASTM A325 Structural Bolts for Construction</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/exploring-astm-a325-structural-bolts-for-construction</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>exploring-astm-a325-structural-bolts-for-construction</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Understanding ASTM F3125 High-Strength Structural Bolts</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/understanding-astm-f3125-high-strength-structural-bolts</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>understanding-astm-f3125-high-strength-structural-bolts</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Understanding ASTM A307 Bolts: Grades and Applications  (note: URL slug references A194 nuts)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/the-essential-guide-to-astm-a194-nuts-l6hkp</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>the-essential-guide-to-astm-a194-nuts-l6hkp</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>The Essential Guide to U-Bolts: Types, Materials, and Applications</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/the-essential-guide-to-u-bolts-types-materials-and-applications</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>the-essential-guide-to-u-bolts-types-materials-and-applications</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Material Selection Spotlight: Nickel Alloy</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/material-selection-spotlight-nickel-alloy</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>material-selection-spotlight-nickel-alloy</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Selecting Fasteners for Extreme Environments</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/choosing-the-right-fasteners-for-extreme-environments</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>choosing-the-right-fasteners-for-extreme-environments</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Seismic-Resistant Fasteners: Choosing the Right Fastener for Earthquake Zones</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/how-to-choose-the-right-fastener-for-seismic-zones</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>how-to-choose-the-right-fastener-for-seismic-zones</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>The Evolution of Fastening Technology in the Construction Industry</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/the-evolution-of-fastening-technology-in-the-construction-industry</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>the-evolution-of-fastening-technology-in-the-construction-industry</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>How Aerospace Fasteners Resist Fatigue &amp; Vibration</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.californiafastener.com/blog/how-aerospace-fasteners-resist-fatigue-vibration</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>how-aerospace-fasteners-resist-fatigue-vibration</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -632,16 +1015,114 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="95" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>New URL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Understanding ASTM A193 B7 vs. A193 B16: A Comprehensive Guide</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://californiafastener.com/blog/astm-a193-b7-vs-a193-b16</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>astm-a193-b7-vs-a193-b16</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>The Ultimate Guide to ASTM F593 Stainless Steel Fasteners</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://californiafastener.com/blog/guide-to-astm-f593-stainless-steel-fasteners</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>guide-to-astm-f593-stainless-steel-fasteners</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>California Fastener — Blog Database &amp; Redirects</t>
+          <t>California Fastener — Blog Migration Database</t>
         </is>
       </c>
     </row>
@@ -651,93 +1132,118 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Source: live site (pulled from the deployed /blog index). 2 published posts.</t>
+          <t>Sheet 1 = posts on the CURRENT live site (www.californiafastener.com/blog, Squarespace).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Sheet 2 = posts already rebuilt on the NEW site (in Sanity CMS).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>New live URLs (your blog lives at /blog/&lt;slug&gt;):</t>
-        </is>
-      </c>
+      <c r="A5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  https://californiafastener.com/blog/astm-a193-b7-vs-a193-b16</t>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>IMPORTANT — completeness:</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  https://californiafastener.com/blog/guide-to-astm-f593-stainless-steel-fasteners</t>
+          <t>The Squarespace site blocks automated access (sitemap/RSS/pages all return 403),</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>so Sheet 1 was compiled from search-engine indexing. It lists 22 posts but may</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Redirects:</t>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>not be 100% complete. For the definitive full list, in a browser open:</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>• If the OLD site's blog used different URLs, fill the 'OLD site URL' column</t>
+          <t xml:space="preserve">   https://www.californiafastener.com/blog?format=json-pretty</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  with each old link. Send it back and I'll add 301 redirects (old → new)</t>
+          <t xml:space="preserve">   (Squarespace's JSON feed lists every post), or check the Squarespace</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  in the site config so existing links/Google results don't 404.</t>
+          <t xml:space="preserve">   dashboard → Pages → Blog. Send me any I'm missing and I'll add them.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>• If the old blog already used /blog/&lt;same-slug&gt;, no redirect is needed —</t>
-        </is>
-      </c>
+      <c r="A13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  the new site serves the same paths.</t>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Redirects:</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Only 1 old post clearly maps to a new one so far (ASTM F593 — the new slug</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Full content (body text, images) lives in the Sanity CMS, editable at</t>
+          <t>differs, so it NEEDS a 301). The rest aren't rebuilt on the new site yet.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  https://californiafastener.com/studio</t>
+          <t>For each old post, fill the yellow 'Redirect → new URL' column with where it</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>should go (the matching new post once created, a related page, or /blog).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Send it back and I'll add the 301 redirects in the site config so old links</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>and Google results don't 404 after the domain cuts over.</t>
         </is>
       </c>
     </row>

</xml_diff>